<commit_message>
Checkpoint teaching decks, assessments and holiday camp materials
</commit_message>
<xml_diff>
--- a/DataAnalysis_Track/DataAnalysis_Track_Workbook.xlsx
+++ b/DataAnalysis_Track/DataAnalysis_Track_Workbook.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Session grid" sheetId="1" state="visible" r:id="rId3"/>
@@ -272,7 +272,7 @@
     <t xml:space="preserve">From notebook to finding. Eleven observations become five findings by striking anything about the data rather than the business, merging duplicates, and ranking what is left by what somebody could do about it. Then the limitation beside each one.</t>
   </si>
   <si>
-    <t xml:space="preserve">Run the routine on the sector dataset you chose: banking and telecom, energy and manufacturing, or public sector and health. Five findings with numbers. This is the mid-track assessment and it is marked on the findings, not the code.</t>
+    <t xml:space="preserve">Run the routine on the sector dataset you chose: banking and telecom, energy and manufacturing, or public sector and development. Use the fixed Bank Marketing, synthetic AI4I or Uganda GDP snapshot. Five findings with numbers. This is the sector assessment and it is marked on the findings, not the code.</t>
   </si>
   <si>
     <t xml:space="preserve">Power BI</t>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">Power BI is three products people confuse: Power Query gets and shapes, the model relates, the report shows. Get Data from CSV, then Power Query: promote headers, set types, trim, remove duplicates. The Applied Steps list as the same idea as the cleaning log from session 8.</t>
   </si>
   <si>
-    <t xml:space="preserve">The model, which is where the marks are. The star schema figure, then five relationships built by hand after deleting every one Power BI guessed. A deliberately wrong relationship first, so the wrong total is seen before the rule is stated. Then the date table, and marking it.</t>
+    <t xml:space="preserve">The model: orders links order_items to customers and reps. Inspect the four relationships built by hand after deleting every one Power BI guessed. A deliberately wrong relationship first, so the wrong total is seen before the rule is stated. Then the date table, and marking it.</t>
   </si>
   <si>
     <t xml:space="preserve">Load the course data, build the model, and produce three visuals whose totals match the numbers you already got in SQL and in pandas. Matching is the mark.</t>
@@ -305,7 +305,7 @@
     <t xml:space="preserve">Design for thirty seconds: the number they came for top left, no more than five visuals, one accent colour, one slicer, and a title that states the finding. Then the five-minute presentation structure: the question, the answer with its number, how you know, what you traded, and what would change your answer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Finish the dashboard, then present. Five minutes each plus questions from the room, and everybody asks at least one question of somebody else. Then twenty minutes on the one report you will replace at work this month.</t>
+    <t xml:space="preserve">Finish the dashboard in 50 minutes. Submit a five-minute narrated presentation. The final hour contains selected demonstrations and 20 minutes on applying the analysis at work.</t>
   </si>
   <si>
     <t xml:space="preserve">The three-hour block</t>
@@ -395,7 +395,7 @@
     <t xml:space="preserve">The same report in pandas, reconciled against the SQL, with the log that makes the starting numbers reproducible. Marked on the log as much as the answer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mid-track investigation</t>
+    <t xml:space="preserve">Sector investigation</t>
   </si>
   <si>
     <t xml:space="preserve">Session 13</t>
@@ -410,7 +410,7 @@
     <t xml:space="preserve">Session 15</t>
   </si>
   <si>
-    <t xml:space="preserve">A dashboard whose totals reconcile, one page of recommendation, and five minutes in front of the room. Marked on whether a decision maker could act on it.</t>
+    <t xml:space="preserve">A dashboard whose totals reconcile, one page of recommendation, and a five-minute presentation with narration in speaker notes. Marked on whether a decision maker could act on it.</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -512,7 +512,7 @@
     <t xml:space="preserve">bank-full.csv is 45,211 rows x 17; bank-additional-full.csv is 41,188 rows x 21. They are different files: say which one.</t>
   </si>
   <si>
-    <t xml:space="preserve">Banking, finance and telecom capstone. Campaign contacts against an outcome, so it carries segmentation, rates and cross-tabs. The duration column leaks the outcome and must be dropped, which makes it a good lesson about leakage.</t>
+    <t xml:space="preserve">Banking, finance and telecom capstone. Campaign contacts against an outcome, so it carries segmentation, rates and cross-tabs. Call duration is known only after the call, so it must not justify pre-call targeting decisions.</t>
   </si>
   <si>
     <t xml:space="preserve">AI4I 2020 Predictive Maintenance (UCI 601)</t>
@@ -524,7 +524,7 @@
     <t xml:space="preserve">10,000 rows x 14 columns, one CSV. Failures are about 3.4% of rows</t>
   </si>
   <si>
-    <t xml:space="preserve">Energy, mining and manufacturing capstone. Machine sensor readings against a failure flag. The imbalance is the point: a rule that predicts no failure is 96.6% accurate and useless.</t>
+    <t xml:space="preserve">Energy, mining and manufacturing capstone. Synthetic machine observations against a failure flag. The imbalance is the point: a rule that predicts no failure is 96.6% accurate and useless.</t>
   </si>
   <si>
     <t xml:space="preserve">World Bank Open Data indicators API</t>
@@ -881,7 +881,7 @@
     <t xml:space="preserve">Date table</t>
   </si>
   <si>
-    <t xml:space="preserve">A separate table with one row per date. Without one, your months sort alphabetically.</t>
+    <t xml:space="preserve">A table with one row per date for consistent time filtering. Sort month names by month number.</t>
   </si>
   <si>
     <t xml:space="preserve">DAX</t>
@@ -1602,96 +1602,100 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1950,502 +1954,502 @@
   <dimension ref="A1:I19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="1" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="6" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="6" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="I16" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="5" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="85.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="5" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2472,156 +2476,156 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <f aca="false">A5</f>
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <f aca="false">B5+A6</f>
         <v>60</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <f aca="false">B6+A7</f>
         <v>70</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <f aca="false">B7+A8</f>
         <v>115</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <f aca="false">B8+A9</f>
         <v>120</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <f aca="false">B9+A10</f>
         <v>170</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <f aca="false">B10+A11</f>
         <v>180</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <f aca="false">SUM(A5:A11)</f>
         <v>180</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="6" t="s">
+      <c r="B12" s="8"/>
+      <c r="C12" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="7"/>
+      <c r="D12" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2646,108 +2650,108 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>0.3</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.4</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <f aca="false">SUM(B5:B8)</f>
         <v>1</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2772,486 +2776,486 @@
   <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <f aca="false">SUM(C5:F5)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="15" t="n">
         <v>75</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="16" t="n">
         <f aca="false">IF(COUNT(C6:F6)=0,"",SUMPRODUCT(C6:F6,C$5:F$5)/SUMPRODUCT((C6:F6&lt;&gt;"")*(C$5:F$5)))</f>
         <v>73.2</v>
       </c>
-      <c r="H6" s="16" t="str">
+      <c r="H6" s="17" t="str">
         <f aca="false">IF(G6="","",IF(G6&gt;=70,"Distinction",IF(G6&gt;=50,"Pass","Not yet")))</f>
         <v>Distinction</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="15" t="str">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="16" t="str">
         <f aca="false">IF(COUNT(C7:F7)=0,"",SUMPRODUCT(C7:F7,C$5:F$5)/SUMPRODUCT((C7:F7&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H7" s="16" t="str">
+      <c r="H7" s="17" t="str">
         <f aca="false">IF(G7="","",IF(G7&gt;=70,"Distinction",IF(G7&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="15" t="str">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="16" t="str">
         <f aca="false">IF(COUNT(C8:F8)=0,"",SUMPRODUCT(C8:F8,C$5:F$5)/SUMPRODUCT((C8:F8&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H8" s="16" t="str">
+      <c r="H8" s="17" t="str">
         <f aca="false">IF(G8="","",IF(G8&gt;=70,"Distinction",IF(G8&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="15" t="str">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="16" t="str">
         <f aca="false">IF(COUNT(C9:F9)=0,"",SUMPRODUCT(C9:F9,C$5:F$5)/SUMPRODUCT((C9:F9&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H9" s="16" t="str">
+      <c r="H9" s="17" t="str">
         <f aca="false">IF(G9="","",IF(G9&gt;=70,"Distinction",IF(G9&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="15" t="str">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="16" t="str">
         <f aca="false">IF(COUNT(C10:F10)=0,"",SUMPRODUCT(C10:F10,C$5:F$5)/SUMPRODUCT((C10:F10&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H10" s="16" t="str">
+      <c r="H10" s="17" t="str">
         <f aca="false">IF(G10="","",IF(G10&gt;=70,"Distinction",IF(G10&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="15" t="str">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="16" t="str">
         <f aca="false">IF(COUNT(C11:F11)=0,"",SUMPRODUCT(C11:F11,C$5:F$5)/SUMPRODUCT((C11:F11&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H11" s="16" t="str">
+      <c r="H11" s="17" t="str">
         <f aca="false">IF(G11="","",IF(G11&gt;=70,"Distinction",IF(G11&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="15" t="str">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="16" t="str">
         <f aca="false">IF(COUNT(C12:F12)=0,"",SUMPRODUCT(C12:F12,C$5:F$5)/SUMPRODUCT((C12:F12&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H12" s="16" t="str">
+      <c r="H12" s="17" t="str">
         <f aca="false">IF(G12="","",IF(G12&gt;=70,"Distinction",IF(G12&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="15" t="str">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="16" t="str">
         <f aca="false">IF(COUNT(C13:F13)=0,"",SUMPRODUCT(C13:F13,C$5:F$5)/SUMPRODUCT((C13:F13&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H13" s="16" t="str">
+      <c r="H13" s="17" t="str">
         <f aca="false">IF(G13="","",IF(G13&gt;=70,"Distinction",IF(G13&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="15" t="str">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="16" t="str">
         <f aca="false">IF(COUNT(C14:F14)=0,"",SUMPRODUCT(C14:F14,C$5:F$5)/SUMPRODUCT((C14:F14&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H14" s="16" t="str">
+      <c r="H14" s="17" t="str">
         <f aca="false">IF(G14="","",IF(G14&gt;=70,"Distinction",IF(G14&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="15" t="str">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="16" t="str">
         <f aca="false">IF(COUNT(C15:F15)=0,"",SUMPRODUCT(C15:F15,C$5:F$5)/SUMPRODUCT((C15:F15&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H15" s="16" t="str">
+      <c r="H15" s="17" t="str">
         <f aca="false">IF(G15="","",IF(G15&gt;=70,"Distinction",IF(G15&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="15" t="str">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="16" t="str">
         <f aca="false">IF(COUNT(C16:F16)=0,"",SUMPRODUCT(C16:F16,C$5:F$5)/SUMPRODUCT((C16:F16&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H16" s="16" t="str">
+      <c r="H16" s="17" t="str">
         <f aca="false">IF(G16="","",IF(G16&gt;=70,"Distinction",IF(G16&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="15" t="str">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="16" t="str">
         <f aca="false">IF(COUNT(C17:F17)=0,"",SUMPRODUCT(C17:F17,C$5:F$5)/SUMPRODUCT((C17:F17&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H17" s="16" t="str">
+      <c r="H17" s="17" t="str">
         <f aca="false">IF(G17="","",IF(G17&gt;=70,"Distinction",IF(G17&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="15" t="str">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="16" t="str">
         <f aca="false">IF(COUNT(C18:F18)=0,"",SUMPRODUCT(C18:F18,C$5:F$5)/SUMPRODUCT((C18:F18&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H18" s="16" t="str">
+      <c r="H18" s="17" t="str">
         <f aca="false">IF(G18="","",IF(G18&gt;=70,"Distinction",IF(G18&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="15" t="str">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="16" t="str">
         <f aca="false">IF(COUNT(C19:F19)=0,"",SUMPRODUCT(C19:F19,C$5:F$5)/SUMPRODUCT((C19:F19&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H19" s="16" t="str">
+      <c r="H19" s="17" t="str">
         <f aca="false">IF(G19="","",IF(G19&gt;=70,"Distinction",IF(G19&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="15" t="str">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="16" t="str">
         <f aca="false">IF(COUNT(C20:F20)=0,"",SUMPRODUCT(C20:F20,C$5:F$5)/SUMPRODUCT((C20:F20&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H20" s="16" t="str">
+      <c r="H20" s="17" t="str">
         <f aca="false">IF(G20="","",IF(G20&gt;=70,"Distinction",IF(G20&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="15" t="str">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="16" t="str">
         <f aca="false">IF(COUNT(C21:F21)=0,"",SUMPRODUCT(C21:F21,C$5:F$5)/SUMPRODUCT((C21:F21&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H21" s="16" t="str">
+      <c r="H21" s="17" t="str">
         <f aca="false">IF(G21="","",IF(G21&gt;=70,"Distinction",IF(G21&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="15" t="str">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="16" t="str">
         <f aca="false">IF(COUNT(C22:F22)=0,"",SUMPRODUCT(C22:F22,C$5:F$5)/SUMPRODUCT((C22:F22&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H22" s="16" t="str">
+      <c r="H22" s="17" t="str">
         <f aca="false">IF(G22="","",IF(G22&gt;=70,"Distinction",IF(G22&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="15" t="str">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="16" t="str">
         <f aca="false">IF(COUNT(C23:F23)=0,"",SUMPRODUCT(C23:F23,C$5:F$5)/SUMPRODUCT((C23:F23&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H23" s="16" t="str">
+      <c r="H23" s="17" t="str">
         <f aca="false">IF(G23="","",IF(G23&gt;=70,"Distinction",IF(G23&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="15" t="str">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="16" t="str">
         <f aca="false">IF(COUNT(C24:F24)=0,"",SUMPRODUCT(C24:F24,C$5:F$5)/SUMPRODUCT((C24:F24&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H24" s="16" t="str">
+      <c r="H24" s="17" t="str">
         <f aca="false">IF(G24="","",IF(G24&gt;=70,"Distinction",IF(G24&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="15" t="str">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="16" t="str">
         <f aca="false">IF(COUNT(C25:F25)=0,"",SUMPRODUCT(C25:F25,C$5:F$5)/SUMPRODUCT((C25:F25&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H25" s="16" t="str">
+      <c r="H25" s="17" t="str">
         <f aca="false">IF(G25="","",IF(G25&gt;=70,"Distinction",IF(G25&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="15" t="str">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="16" t="str">
         <f aca="false">IF(COUNT(C26:F26)=0,"",SUMPRODUCT(C26:F26,C$5:F$5)/SUMPRODUCT((C26:F26&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H26" s="16" t="str">
+      <c r="H26" s="17" t="str">
         <f aca="false">IF(G26="","",IF(G26&gt;=70,"Distinction",IF(G26&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="15" t="str">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="16" t="str">
         <f aca="false">IF(COUNT(C27:F27)=0,"",SUMPRODUCT(C27:F27,C$5:F$5)/SUMPRODUCT((C27:F27&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H27" s="16" t="str">
+      <c r="H27" s="17" t="str">
         <f aca="false">IF(G27="","",IF(G27&gt;=70,"Distinction",IF(G27&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="15" t="str">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="16" t="str">
         <f aca="false">IF(COUNT(C28:F28)=0,"",SUMPRODUCT(C28:F28,C$5:F$5)/SUMPRODUCT((C28:F28&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H28" s="16" t="str">
+      <c r="H28" s="17" t="str">
         <f aca="false">IF(G28="","",IF(G28&gt;=70,"Distinction",IF(G28&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="15" t="str">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="16" t="str">
         <f aca="false">IF(COUNT(C29:F29)=0,"",SUMPRODUCT(C29:F29,C$5:F$5)/SUMPRODUCT((C29:F29&lt;&gt;"")*(C$5:F$5)))</f>
         <v/>
       </c>
-      <c r="H29" s="16" t="str">
+      <c r="H29" s="17" t="str">
         <f aca="false">IF(G29="","",IF(G29&gt;=70,"Distinction",IF(G29&gt;=50,"Pass","Not yet")))</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="19" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3278,243 +3282,243 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3545,214 +3549,214 @@
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>6000</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>4837</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>575</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>6000</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>5828</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="22" t="n">
         <v>10758894480</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <v>8751705520</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="22" t="n">
         <v>390632335</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="6" t="n">
         <v>172</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="22" t="n">
         <v>197830550</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="22" t="n">
         <v>8751672145.42</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <v>33374.58</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <v>1793149.08</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="B18" s="21" t="n">
+      <c r="B18" s="22" t="n">
         <v>374760</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="6" t="n">
         <v>4.785</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="B20" s="21" t="n">
+      <c r="B20" s="22" t="n">
         <v>3896620</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="19" t="s">
         <v>223</v>
       </c>
     </row>
@@ -3779,1332 +3783,1332 @@
   <dimension ref="A1:D98"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D22" s="5" t="n">
+      <c r="D22" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D23" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D27" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D28" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D31" s="5" t="n">
+      <c r="D31" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D32" s="5" t="n">
+      <c r="D32" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="C33" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D33" s="5" t="n">
+      <c r="D33" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D34" s="5" t="n">
+      <c r="D34" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="C35" s="22" t="s">
+      <c r="C35" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D35" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D36" s="5" t="n">
+      <c r="D36" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="D37" s="5" t="n">
+      <c r="D37" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="C38" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="D38" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="D39" s="5" t="n">
+      <c r="D39" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="D40" s="5" t="n">
+      <c r="D40" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="D41" s="5" t="n">
+      <c r="D41" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D42" s="5" t="n">
+      <c r="D42" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="C43" s="22" t="s">
+      <c r="C43" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D43" s="5" t="n">
+      <c r="D43" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="D44" s="5" t="n">
+      <c r="D44" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="D45" s="5" t="n">
+      <c r="D45" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D46" s="5" t="n">
+      <c r="D46" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="D47" s="5" t="n">
+      <c r="D47" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="D48" s="5" t="n">
+      <c r="D48" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="C49" s="22" t="s">
+      <c r="C49" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D49" s="5" t="n">
+      <c r="D49" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="C50" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D50" s="5" t="n">
+      <c r="D50" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="D51" s="5" t="n">
+      <c r="D51" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
+      <c r="A52" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="D52" s="5" t="n">
+      <c r="D52" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="D53" s="5" t="n">
+      <c r="D53" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="D54" s="5" t="n">
+      <c r="D54" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="D55" s="5" t="n">
+      <c r="D55" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="5" t="s">
+      <c r="A56" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="D56" s="5" t="n">
+      <c r="D56" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5" t="s">
+      <c r="A57" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="C57" s="22" t="s">
+      <c r="C57" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D57" s="5" t="n">
+      <c r="D57" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
+      <c r="A58" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="D58" s="5" t="n">
+      <c r="D58" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="C59" s="22" t="s">
+      <c r="C59" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D59" s="5" t="n">
+      <c r="D59" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="C60" s="22" t="s">
+      <c r="C60" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D60" s="5" t="n">
+      <c r="D60" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="D61" s="5" t="n">
+      <c r="D61" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="C62" s="22" t="s">
+      <c r="C62" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D62" s="5" t="n">
+      <c r="D62" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="C63" s="22" t="s">
+      <c r="C63" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D63" s="5" t="n">
+      <c r="D63" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D64" s="5" t="n">
+      <c r="D64" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="D65" s="5" t="n">
+      <c r="D65" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="C66" s="22" t="s">
+      <c r="C66" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D66" s="5" t="n">
+      <c r="D66" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="s">
+      <c r="A67" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="C67" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="D67" s="5" t="n">
+      <c r="D67" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="C68" s="22" t="s">
+      <c r="C68" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D68" s="5" t="n">
+      <c r="D68" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
+      <c r="A69" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C69" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="D69" s="5" t="n">
+      <c r="D69" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="5" t="s">
+      <c r="A70" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="C70" s="22" t="s">
+      <c r="C70" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D70" s="5" t="n">
+      <c r="D70" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="5" t="s">
+      <c r="A71" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="C71" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="D71" s="5" t="n">
+      <c r="D71" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="5" t="s">
+      <c r="A72" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="B72" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="C72" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="D72" s="5" t="n">
+      <c r="D72" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="C73" s="22" t="s">
+      <c r="C73" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D73" s="5" t="n">
+      <c r="D73" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="C74" s="22" t="s">
+      <c r="C74" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D74" s="5" t="n">
+      <c r="D74" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="5" t="s">
+      <c r="A75" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="B75" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="C75" s="22" t="s">
+      <c r="C75" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D75" s="5" t="n">
+      <c r="D75" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="B76" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="C76" s="22" t="s">
+      <c r="C76" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D76" s="5" t="n">
+      <c r="D76" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="C77" s="22" t="s">
+      <c r="C77" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D77" s="5" t="n">
+      <c r="D77" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="C78" s="5" t="s">
+      <c r="C78" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="D78" s="5" t="n">
+      <c r="D78" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="5" t="s">
+      <c r="A79" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="C79" s="22" t="s">
+      <c r="C79" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D79" s="5" t="n">
+      <c r="D79" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="5" t="s">
+      <c r="A80" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="C80" s="22" t="s">
+      <c r="C80" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D80" s="5" t="n">
+      <c r="D80" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="5" t="s">
+      <c r="A81" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="C81" s="22" t="s">
+      <c r="C81" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D81" s="5" t="n">
+      <c r="D81" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="5" t="s">
+      <c r="A82" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="B82" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="C82" s="22" t="s">
+      <c r="C82" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D82" s="5" t="n">
+      <c r="D82" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="5" t="s">
+      <c r="A83" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="B83" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="C83" s="5" t="s">
+      <c r="C83" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="D83" s="5" t="n">
+      <c r="D83" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="C84" s="22" t="s">
+      <c r="C84" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D84" s="5" t="n">
+      <c r="D84" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="5" t="s">
+      <c r="A85" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="B85" s="5" t="s">
+      <c r="B85" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="C85" s="22" t="s">
+      <c r="C85" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D85" s="5" t="n">
+      <c r="D85" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="5" t="s">
+      <c r="A86" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="B86" s="5" t="s">
+      <c r="B86" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="D86" s="5" t="n">
+      <c r="D86" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="5" t="s">
+      <c r="A87" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="C87" s="22" t="s">
+      <c r="C87" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D87" s="5" t="n">
+      <c r="D87" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="5" t="s">
+      <c r="A88" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="C88" s="5" t="s">
+      <c r="C88" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="D88" s="5" t="n">
+      <c r="D88" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="5" t="s">
+      <c r="A89" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="B89" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="C89" s="22" t="s">
+      <c r="C89" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D89" s="5" t="n">
+      <c r="D89" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="5" t="s">
+      <c r="A90" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="B90" s="5" t="s">
+      <c r="B90" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="C90" s="22" t="s">
+      <c r="C90" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D90" s="5" t="n">
+      <c r="D90" s="6" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
+      <c r="A91" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="B91" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="C91" s="22" t="s">
+      <c r="C91" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D91" s="5" t="n">
+      <c r="D91" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="B92" s="5" t="s">
+      <c r="B92" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="C92" s="22" t="s">
+      <c r="C92" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D92" s="5" t="n">
+      <c r="D92" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="5" t="s">
+      <c r="A93" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="B93" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="C93" s="5" t="s">
+      <c r="C93" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="D93" s="5" t="n">
+      <c r="D93" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="B94" s="5" t="s">
+      <c r="B94" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="D94" s="5" t="n">
+      <c r="D94" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="5" t="s">
+      <c r="A95" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="B95" s="5" t="s">
+      <c r="B95" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="C95" s="22" t="s">
+      <c r="C95" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D95" s="5" t="n">
+      <c r="D95" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="5" t="s">
+      <c r="A96" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="B96" s="5" t="s">
+      <c r="B96" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="C96" s="22" t="s">
+      <c r="C96" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="D96" s="5" t="n">
+      <c r="D96" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="18" t="s">
+      <c r="A98" s="19" t="s">
         <v>456</v>
       </c>
     </row>
@@ -5131,59 +5135,59 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>467</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>468</v>
       </c>
     </row>

</xml_diff>